<commit_message>
data(pscboxdia): S15 하부 헌치를 한 단으로 — WBHUL2 0
도면의 하부슬래브 헌치는 복부 내면에서 한 번에 내려오는 한 단이다. 그것을
875 + 875 두 구간으로 쪼개고 중간 두께 925 를 지어내 적고 있었다. 직선 위의
점이라 형상은 같았지만, 도면에 없는 꺾임점을 입력이 주장하는 셈이었다.

  WBHUL1  875 → 1750   복부 내면(-3,000)에서 -1,250 까지 한 번에
  TBHL2   925 → 800    꺾이는 자리의 두께 = TBS
  WBHUL2  875 → 0      둘째 구간 없음

검증 : 도면 8-018 에서 실측한 절점 17개가 그대로 일치. PBHL2 가 PBHL3 와 한
점이 되고(-1250, -6962.5), 길이 0 세그먼트는 벽을 만들지 않아 벽이 36 → 34,
zeroLen 0. 고리는 여전히 [외곽 14, 셀 12, 개구부 8] 로 각각 닫힌다.

상부 헌치(WTHUL1/2 875+875)도 도면상 한 단이지만 이번에는 손대지 않았다.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pxd9b9G4a1bcy9FpZN9nhs
</commit_message>
<xml_diff>
--- a/PSCBOX_DIAPHRAGM_S15.xlsx
+++ b/PSCBOX_DIAPHRAGM_S15.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K58"/>
+  <dimension ref="A1:J58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -916,7 +916,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t># ---- bottom slab haunch : 1,050 at the web -&gt; 800 over a 1,750 run ----</t>
+          <t># ---- bottom slab haunch : one step, 1,050 at the web -&gt; 800 over a 1,750 run ----</t>
         </is>
       </c>
       <c r="C40" s="2" t="n"/>
@@ -948,7 +948,12 @@
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>925</v>
+        <v>800</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>same as TBS — the haunch ends here</t>
+        </is>
       </c>
     </row>
     <row r="43">
@@ -963,7 +968,7 @@
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>875</v>
+        <v>1750</v>
       </c>
     </row>
     <row r="44">
@@ -978,7 +983,12 @@
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>875</v>
+        <v>0</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>one-step haunch: the second run is not used</t>
+        </is>
       </c>
     </row>
     <row r="45">

</xml_diff>

<commit_message>
data(pscboxdia): S15 상부 헌치도 한 단으로 — WTHUL2 0
하부와 같은 이유다. 도면의 상부슬래브 헌치는 복부 내면에서 한 번에 내려오는
한 단인데 875 + 875 로 쪼개고 중간 두께 440 을 지어내 적고 있었다.

  WTHUL1  875 → 1750   복부 내면(∓3,000)에서 ∓1,250 까지 한 번에
  TTHL2   440 → 280    꺾이는 자리의 두께 = TTS
  WTHUL2  875 → 0      둘째 구간 없음

검증 : 절점 17개 그대로 일치. 상·하 네 헌치의 중간점이 모두 끝점과 한 점이
되고(PTHL2=PTHL3, PTHR2=PTHR3, PBHL2=PBHL3, PBHR2=PBHR3), 벽이 34 → 32,
zeroLen 0, 고리 [외곽 14, 셀 10, 개구부 8] 로 각각 닫힌다.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pxd9b9G4a1bcy9FpZN9nhs
</commit_message>
<xml_diff>
--- a/PSCBOX_DIAPHRAGM_S15.xlsx
+++ b/PSCBOX_DIAPHRAGM_S15.xlsx
@@ -845,7 +845,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t># ---- top slab haunch : 600 at the web -&gt; 280 over a 1,750 run ----</t>
+          <t># ---- top slab haunch : one step, 600 at the web -&gt; 280 over a 1,750 run ----</t>
         </is>
       </c>
       <c r="C34" s="2" t="n"/>
@@ -877,7 +877,12 @@
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>440</v>
+        <v>280</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>same as TTS — the haunch ends here</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -892,7 +897,7 @@
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>875</v>
+        <v>1750</v>
       </c>
     </row>
     <row r="38">
@@ -907,7 +912,12 @@
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>875</v>
+        <v>0</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>one-step haunch: the second run is not used</t>
+        </is>
       </c>
     </row>
     <row r="39">

</xml_diff>